<commit_message>
Error Fixed of UI
</commit_message>
<xml_diff>
--- a/BI_Analysis_Report_2026.xlsx
+++ b/BI_Analysis_Report_2026.xlsx
@@ -1786,22 +1786,55 @@
       <c r="B30" s="2" t="n">
         <v>46291</v>
       </c>
-      <c r="C30" s="1" t="n"/>
-      <c r="D30" s="1" t="n"/>
-      <c r="E30" s="1" t="n"/>
-      <c r="F30" s="1" t="n"/>
-      <c r="G30" s="1" t="n"/>
-      <c r="H30" s="1" t="n"/>
-      <c r="I30" s="1" t="n"/>
-      <c r="J30" s="1" t="n"/>
-      <c r="K30" s="1" t="n"/>
-      <c r="L30" s="1" t="n"/>
-      <c r="M30" s="1" t="n"/>
-      <c r="N30" s="1" t="n"/>
-      <c r="O30" s="1" t="n"/>
-      <c r="P30" s="1" t="n"/>
-      <c r="Q30" s="1" t="n"/>
-      <c r="R30" s="1" t="n"/>
+      <c r="C30" s="11" t="n">
+        <v>3306.11</v>
+      </c>
+      <c r="D30" s="11" t="n">
+        <v>104.4</v>
+      </c>
+      <c r="E30" s="11" t="n">
+        <v>461.67</v>
+      </c>
+      <c r="F30" s="11" t="n">
+        <v>128.19</v>
+      </c>
+      <c r="G30" s="11" t="n">
+        <v>1113.45</v>
+      </c>
+      <c r="H30" s="11" t="n">
+        <v>1996.49</v>
+      </c>
+      <c r="I30" s="11" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="J30" s="11" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="K30" s="11" t="n">
+        <v>784.3099999999999</v>
+      </c>
+      <c r="L30" s="11" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="M30" s="11" t="n">
+        <v>1013.04</v>
+      </c>
+      <c r="N30" s="11" t="n">
+        <v>21.24</v>
+      </c>
+      <c r="O30" s="11" t="n">
+        <v>726.8099999999999</v>
+      </c>
+      <c r="P30" s="11" t="n">
+        <v>657.91</v>
+      </c>
+      <c r="Q30" s="11" t="n">
+        <v>171.91</v>
+      </c>
+      <c r="R30" s="11">
+        <f>SUM(C30:Q30)</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="B31" s="2" t="n">

</xml_diff>

<commit_message>
Excel Sheet Updated 21-10-2026
</commit_message>
<xml_diff>
--- a/BI_Analysis_Report_2026.xlsx
+++ b/BI_Analysis_Report_2026.xlsx
@@ -1840,22 +1840,55 @@
       <c r="B31" s="2" t="n">
         <v>46292</v>
       </c>
-      <c r="C31" s="1" t="n"/>
-      <c r="D31" s="1" t="n"/>
-      <c r="E31" s="1" t="n"/>
-      <c r="F31" s="1" t="n"/>
-      <c r="G31" s="1" t="n"/>
-      <c r="H31" s="1" t="n"/>
-      <c r="I31" s="1" t="n"/>
-      <c r="J31" s="1" t="n"/>
-      <c r="K31" s="1" t="n"/>
-      <c r="L31" s="1" t="n"/>
-      <c r="M31" s="1" t="n"/>
-      <c r="N31" s="1" t="n"/>
-      <c r="O31" s="1" t="n"/>
-      <c r="P31" s="1" t="n"/>
-      <c r="Q31" s="1" t="n"/>
-      <c r="R31" s="1" t="n"/>
+      <c r="C31" s="11" t="n">
+        <v>3276.92</v>
+      </c>
+      <c r="D31" s="11" t="n">
+        <v>81.83</v>
+      </c>
+      <c r="E31" s="11" t="n">
+        <v>521.87</v>
+      </c>
+      <c r="F31" s="11" t="n">
+        <v>151.71</v>
+      </c>
+      <c r="G31" s="11" t="n">
+        <v>995.4</v>
+      </c>
+      <c r="H31" s="11" t="n">
+        <v>2059.25</v>
+      </c>
+      <c r="I31" s="11" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J31" s="11" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="K31" s="11" t="n">
+        <v>790.88</v>
+      </c>
+      <c r="L31" s="11" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="M31" s="11" t="n">
+        <v>990.29</v>
+      </c>
+      <c r="N31" s="11" t="n">
+        <v>18.43</v>
+      </c>
+      <c r="O31" s="11" t="n">
+        <v>736.91</v>
+      </c>
+      <c r="P31" s="11" t="n">
+        <v>690.27</v>
+      </c>
+      <c r="Q31" s="11" t="n">
+        <v>148.55</v>
+      </c>
+      <c r="R31" s="11">
+        <f>SUM(C31:Q31)</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="B32" s="2" t="n">
@@ -2011,421 +2044,1079 @@
       <c r="B36" s="2" t="n">
         <v>46297</v>
       </c>
-      <c r="C36" s="1" t="n"/>
-      <c r="D36" s="1" t="n"/>
-      <c r="E36" s="1" t="n"/>
-      <c r="F36" s="1" t="n"/>
-      <c r="G36" s="1" t="n"/>
-      <c r="H36" s="1" t="n"/>
-      <c r="I36" s="1" t="n"/>
-      <c r="J36" s="1" t="n"/>
-      <c r="K36" s="1" t="n"/>
-      <c r="L36" s="1" t="n"/>
-      <c r="M36" s="1" t="n"/>
-      <c r="N36" s="1" t="n"/>
-      <c r="O36" s="1" t="n"/>
-      <c r="P36" s="1" t="n"/>
-      <c r="Q36" s="1" t="n"/>
-      <c r="R36" s="1" t="n"/>
+      <c r="C36" s="11" t="n">
+        <v>3755.42</v>
+      </c>
+      <c r="D36" s="11" t="n">
+        <v>77.09999999999999</v>
+      </c>
+      <c r="E36" s="11" t="n">
+        <v>507.24</v>
+      </c>
+      <c r="F36" s="11" t="n">
+        <v>129.38</v>
+      </c>
+      <c r="G36" s="11" t="n">
+        <v>1142.53</v>
+      </c>
+      <c r="H36" s="11" t="n">
+        <v>2135.18</v>
+      </c>
+      <c r="I36" s="11" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="J36" s="11" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="K36" s="11" t="n">
+        <v>790.29</v>
+      </c>
+      <c r="L36" s="11" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M36" s="11" t="n">
+        <v>1024.55</v>
+      </c>
+      <c r="N36" s="11" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="O36" s="11" t="n">
+        <v>735.86</v>
+      </c>
+      <c r="P36" s="11" t="n">
+        <v>716.4299999999999</v>
+      </c>
+      <c r="Q36" s="11" t="n">
+        <v>184.62</v>
+      </c>
+      <c r="R36" s="11">
+        <f>SUM(C36:Q36)</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="B37" s="2" t="n">
         <v>46298</v>
       </c>
-      <c r="C37" s="1" t="n"/>
-      <c r="D37" s="1" t="n"/>
-      <c r="E37" s="1" t="n"/>
-      <c r="F37" s="1" t="n"/>
-      <c r="G37" s="1" t="n"/>
-      <c r="H37" s="1" t="n"/>
-      <c r="I37" s="1" t="n"/>
-      <c r="J37" s="1" t="n"/>
-      <c r="K37" s="1" t="n"/>
-      <c r="L37" s="1" t="n"/>
-      <c r="M37" s="1" t="n"/>
+      <c r="C37" s="11" t="n">
+        <v>888.22</v>
+      </c>
+      <c r="D37" s="11" t="n">
+        <v>27.06</v>
+      </c>
+      <c r="E37" s="11" t="n">
+        <v>101.97</v>
+      </c>
+      <c r="F37" s="11" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="G37" s="11" t="n">
+        <v>269.88</v>
+      </c>
+      <c r="H37" s="11" t="n">
+        <v>584.6799999999999</v>
+      </c>
+      <c r="I37" s="11" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J37" s="11" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="K37" s="11" t="n">
+        <v>300.39</v>
+      </c>
+      <c r="L37" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M37" s="11" t="n">
+        <v>162.82</v>
+      </c>
       <c r="N37" s="1" t="n"/>
-      <c r="O37" s="1" t="n"/>
-      <c r="P37" s="1" t="n"/>
-      <c r="Q37" s="1" t="n"/>
-      <c r="R37" s="1" t="n"/>
+      <c r="O37" s="11" t="n">
+        <v>160.67</v>
+      </c>
+      <c r="P37" s="11" t="n">
+        <v>184.42</v>
+      </c>
+      <c r="Q37" s="11" t="n">
+        <v>72.48999999999999</v>
+      </c>
+      <c r="R37" s="11">
+        <f>C37+D37+E37+F37+G37+H37+I37+J37+K37+L37+M37+O37+P37+Q37</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="B38" s="2" t="n">
         <v>46299</v>
       </c>
-      <c r="C38" s="1" t="n"/>
-      <c r="D38" s="1" t="n"/>
-      <c r="E38" s="1" t="n"/>
-      <c r="F38" s="1" t="n"/>
-      <c r="G38" s="1" t="n"/>
-      <c r="H38" s="1" t="n"/>
-      <c r="I38" s="1" t="n"/>
-      <c r="J38" s="1" t="n"/>
-      <c r="K38" s="1" t="n"/>
-      <c r="L38" s="1" t="n"/>
-      <c r="M38" s="1" t="n"/>
-      <c r="N38" s="1" t="n"/>
-      <c r="O38" s="1" t="n"/>
-      <c r="P38" s="1" t="n"/>
-      <c r="Q38" s="1" t="n"/>
-      <c r="R38" s="1" t="n"/>
+      <c r="C38" s="11" t="n">
+        <v>3067.8</v>
+      </c>
+      <c r="D38" s="11" t="n">
+        <v>72.72</v>
+      </c>
+      <c r="E38" s="11" t="n">
+        <v>431.34</v>
+      </c>
+      <c r="F38" s="11" t="n">
+        <v>155.6</v>
+      </c>
+      <c r="G38" s="11" t="n">
+        <v>975.41</v>
+      </c>
+      <c r="H38" s="11" t="n">
+        <v>1631.4</v>
+      </c>
+      <c r="I38" s="11" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="J38" s="11" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="K38" s="11" t="n">
+        <v>592.1799999999999</v>
+      </c>
+      <c r="L38" s="11" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M38" s="11" t="n">
+        <v>834.52</v>
+      </c>
+      <c r="N38" s="11" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="O38" s="11" t="n">
+        <v>551.12</v>
+      </c>
+      <c r="P38" s="11" t="n">
+        <v>505.52</v>
+      </c>
+      <c r="Q38" s="11" t="n">
+        <v>155.04</v>
+      </c>
+      <c r="R38" s="11">
+        <f>SUM(C38:Q38)</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="B39" s="2" t="n">
         <v>46300</v>
       </c>
-      <c r="C39" s="1" t="n"/>
-      <c r="D39" s="1" t="n"/>
-      <c r="E39" s="1" t="n"/>
-      <c r="F39" s="1" t="n"/>
-      <c r="G39" s="1" t="n"/>
-      <c r="H39" s="1" t="n"/>
-      <c r="I39" s="1" t="n"/>
-      <c r="J39" s="1" t="n"/>
-      <c r="K39" s="1" t="n"/>
-      <c r="L39" s="1" t="n"/>
-      <c r="M39" s="1" t="n"/>
-      <c r="N39" s="1" t="n"/>
-      <c r="O39" s="1" t="n"/>
-      <c r="P39" s="1" t="n"/>
-      <c r="Q39" s="1" t="n"/>
-      <c r="R39" s="1" t="n"/>
+      <c r="C39" s="11" t="n">
+        <v>976.64</v>
+      </c>
+      <c r="D39" s="11" t="n">
+        <v>22.92</v>
+      </c>
+      <c r="E39" s="11" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="F39" s="11" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="G39" s="11" t="n">
+        <v>303.84</v>
+      </c>
+      <c r="H39" s="11" t="n">
+        <v>669.17</v>
+      </c>
+      <c r="I39" s="11" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="J39" s="11" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="K39" s="11" t="n">
+        <v>246.8</v>
+      </c>
+      <c r="L39" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M39" s="11" t="n">
+        <v>229.77</v>
+      </c>
+      <c r="N39" s="11" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="O39" s="11" t="n">
+        <v>203.74</v>
+      </c>
+      <c r="P39" s="11" t="n">
+        <v>231.55</v>
+      </c>
+      <c r="Q39" s="11" t="n">
+        <v>94.73999999999999</v>
+      </c>
+      <c r="R39" s="11">
+        <f>SUM(C39:Q39)</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="B40" s="2" t="n">
         <v>46301</v>
       </c>
-      <c r="C40" s="1" t="n"/>
-      <c r="D40" s="1" t="n"/>
-      <c r="E40" s="1" t="n"/>
-      <c r="F40" s="1" t="n"/>
-      <c r="G40" s="1" t="n"/>
-      <c r="H40" s="1" t="n"/>
-      <c r="I40" s="1" t="n"/>
-      <c r="J40" s="1" t="n"/>
-      <c r="K40" s="1" t="n"/>
-      <c r="L40" s="1" t="n"/>
-      <c r="M40" s="1" t="n"/>
-      <c r="N40" s="1" t="n"/>
-      <c r="O40" s="1" t="n"/>
-      <c r="P40" s="1" t="n"/>
-      <c r="Q40" s="1" t="n"/>
-      <c r="R40" s="1" t="n"/>
+      <c r="C40" s="11" t="n">
+        <v>3038.24</v>
+      </c>
+      <c r="D40" s="11" t="n">
+        <v>74.98</v>
+      </c>
+      <c r="E40" s="11" t="n">
+        <v>448.07</v>
+      </c>
+      <c r="F40" s="11" t="n">
+        <v>151.45</v>
+      </c>
+      <c r="G40" s="11" t="n">
+        <v>985.4</v>
+      </c>
+      <c r="H40" s="11" t="n">
+        <v>1574.03</v>
+      </c>
+      <c r="I40" s="11" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="J40" s="11" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="K40" s="11" t="n">
+        <v>596.6</v>
+      </c>
+      <c r="L40" s="11" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M40" s="11" t="n">
+        <v>839.78</v>
+      </c>
+      <c r="N40" s="11" t="n">
+        <v>17.74</v>
+      </c>
+      <c r="O40" s="11" t="n">
+        <v>544.24</v>
+      </c>
+      <c r="P40" s="11" t="n">
+        <v>497.28</v>
+      </c>
+      <c r="Q40" s="11" t="n">
+        <v>158.43</v>
+      </c>
+      <c r="R40" s="11">
+        <f>SUM(C40:Q40)</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="B41" s="2" t="n">
         <v>46302</v>
       </c>
-      <c r="C41" s="1" t="n"/>
-      <c r="D41" s="1" t="n"/>
-      <c r="E41" s="1" t="n"/>
-      <c r="F41" s="1" t="n"/>
-      <c r="G41" s="1" t="n"/>
-      <c r="H41" s="1" t="n"/>
-      <c r="I41" s="1" t="n"/>
-      <c r="J41" s="1" t="n"/>
-      <c r="K41" s="1" t="n"/>
-      <c r="L41" s="1" t="n"/>
-      <c r="M41" s="1" t="n"/>
-      <c r="N41" s="1" t="n"/>
-      <c r="O41" s="1" t="n"/>
-      <c r="P41" s="1" t="n"/>
-      <c r="Q41" s="1" t="n"/>
-      <c r="R41" s="1" t="n"/>
+      <c r="C41" s="11" t="n">
+        <v>3748.32</v>
+      </c>
+      <c r="D41" s="11" t="n">
+        <v>112.84</v>
+      </c>
+      <c r="E41" s="11" t="n">
+        <v>444.91</v>
+      </c>
+      <c r="F41" s="11" t="n">
+        <v>159.77</v>
+      </c>
+      <c r="G41" s="11" t="n">
+        <v>1027.03</v>
+      </c>
+      <c r="H41" s="11" t="n">
+        <v>1972.74</v>
+      </c>
+      <c r="I41" s="11" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="J41" s="11" t="n">
+        <v>44.06</v>
+      </c>
+      <c r="K41" s="11" t="n">
+        <v>781.78</v>
+      </c>
+      <c r="L41" s="11" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="M41" s="11" t="n">
+        <v>1051.4</v>
+      </c>
+      <c r="N41" s="11" t="n">
+        <v>16.22</v>
+      </c>
+      <c r="O41" s="11" t="n">
+        <v>730.42</v>
+      </c>
+      <c r="P41" s="11" t="n">
+        <v>612.17</v>
+      </c>
+      <c r="Q41" s="11" t="n">
+        <v>184.77</v>
+      </c>
+      <c r="R41" s="11">
+        <f>SUM(C41:Q41)</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="B42" s="2" t="n">
         <v>46303</v>
       </c>
-      <c r="C42" s="1" t="n"/>
-      <c r="D42" s="1" t="n"/>
-      <c r="E42" s="1" t="n"/>
-      <c r="F42" s="1" t="n"/>
-      <c r="G42" s="1" t="n"/>
-      <c r="H42" s="1" t="n"/>
-      <c r="I42" s="1" t="n"/>
-      <c r="J42" s="1" t="n"/>
-      <c r="K42" s="1" t="n"/>
-      <c r="L42" s="1" t="n"/>
-      <c r="M42" s="1" t="n"/>
-      <c r="N42" s="1" t="n"/>
-      <c r="O42" s="1" t="n"/>
-      <c r="P42" s="1" t="n"/>
-      <c r="Q42" s="1" t="n"/>
-      <c r="R42" s="1" t="n"/>
+      <c r="C42" s="11" t="n">
+        <v>4205.83</v>
+      </c>
+      <c r="D42" s="11" t="n">
+        <v>130.81</v>
+      </c>
+      <c r="E42" s="11" t="n">
+        <v>534.28</v>
+      </c>
+      <c r="F42" s="11" t="n">
+        <v>203.26</v>
+      </c>
+      <c r="G42" s="11" t="n">
+        <v>1016.07</v>
+      </c>
+      <c r="H42" s="11" t="n">
+        <v>2012.4</v>
+      </c>
+      <c r="I42" s="11" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="J42" s="11" t="n">
+        <v>315.91</v>
+      </c>
+      <c r="K42" s="11" t="n">
+        <v>774.22</v>
+      </c>
+      <c r="L42" s="11" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="M42" s="11" t="n">
+        <v>1037.01</v>
+      </c>
+      <c r="N42" s="11" t="n">
+        <v>14.58</v>
+      </c>
+      <c r="O42" s="11" t="n">
+        <v>733.75</v>
+      </c>
+      <c r="P42" s="11" t="n">
+        <v>637.52</v>
+      </c>
+      <c r="Q42" s="11" t="n">
+        <v>163.04</v>
+      </c>
+      <c r="R42" s="11">
+        <f>SUM(C42:Q42)</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="B43" s="2" t="n">
         <v>46304</v>
       </c>
-      <c r="C43" s="1" t="n"/>
-      <c r="D43" s="1" t="n"/>
-      <c r="E43" s="1" t="n"/>
-      <c r="F43" s="1" t="n"/>
-      <c r="G43" s="1" t="n"/>
-      <c r="H43" s="1" t="n"/>
-      <c r="I43" s="1" t="n"/>
-      <c r="J43" s="1" t="n"/>
-      <c r="K43" s="1" t="n"/>
-      <c r="L43" s="1" t="n"/>
-      <c r="M43" s="1" t="n"/>
-      <c r="N43" s="1" t="n"/>
-      <c r="O43" s="1" t="n"/>
-      <c r="P43" s="1" t="n"/>
-      <c r="Q43" s="1" t="n"/>
-      <c r="R43" s="1" t="n"/>
+      <c r="C43" s="11" t="n">
+        <v>3686.17</v>
+      </c>
+      <c r="D43" s="11" t="n">
+        <v>129.96</v>
+      </c>
+      <c r="E43" s="11" t="n">
+        <v>442.88</v>
+      </c>
+      <c r="F43" s="11" t="n">
+        <v>182.18</v>
+      </c>
+      <c r="G43" s="11" t="n">
+        <v>1087.72</v>
+      </c>
+      <c r="H43" s="11" t="n">
+        <v>1921.2</v>
+      </c>
+      <c r="I43" s="11" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="J43" s="11" t="n">
+        <v>312.31</v>
+      </c>
+      <c r="K43" s="11" t="n">
+        <v>778.46</v>
+      </c>
+      <c r="L43" s="11" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="M43" s="11" t="n">
+        <v>981.11</v>
+      </c>
+      <c r="N43" s="11" t="n">
+        <v>11.95</v>
+      </c>
+      <c r="O43" s="11" t="n">
+        <v>731.6</v>
+      </c>
+      <c r="P43" s="11" t="n">
+        <v>609.7</v>
+      </c>
+      <c r="Q43" s="11" t="n">
+        <v>151.84</v>
+      </c>
+      <c r="R43" s="11">
+        <f>SUM(C43:Q43)</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="B44" s="2" t="n">
         <v>46305</v>
       </c>
-      <c r="C44" s="1" t="n"/>
-      <c r="D44" s="1" t="n"/>
-      <c r="E44" s="1" t="n"/>
-      <c r="F44" s="1" t="n"/>
-      <c r="G44" s="1" t="n"/>
-      <c r="H44" s="1" t="n"/>
-      <c r="I44" s="1" t="n"/>
-      <c r="J44" s="1" t="n"/>
-      <c r="K44" s="1" t="n"/>
-      <c r="L44" s="1" t="n"/>
-      <c r="M44" s="1" t="n"/>
-      <c r="N44" s="1" t="n"/>
-      <c r="O44" s="1" t="n"/>
-      <c r="P44" s="1" t="n"/>
-      <c r="Q44" s="1" t="n"/>
-      <c r="R44" s="1" t="n"/>
+      <c r="C44" s="11" t="n">
+        <v>3627.42</v>
+      </c>
+      <c r="D44" s="11" t="n">
+        <v>120.06</v>
+      </c>
+      <c r="E44" s="11" t="n">
+        <v>425.02</v>
+      </c>
+      <c r="F44" s="11" t="n">
+        <v>123.63</v>
+      </c>
+      <c r="G44" s="11" t="n">
+        <v>1107.28</v>
+      </c>
+      <c r="H44" s="11" t="n">
+        <v>1730.21</v>
+      </c>
+      <c r="I44" s="11" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="J44" s="11" t="n">
+        <v>233.31</v>
+      </c>
+      <c r="K44" s="11" t="n">
+        <v>771.6</v>
+      </c>
+      <c r="L44" s="11" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="M44" s="11" t="n">
+        <v>901.23</v>
+      </c>
+      <c r="N44" s="11" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="O44" s="11" t="n">
+        <v>617.5</v>
+      </c>
+      <c r="P44" s="11" t="n">
+        <v>521.0700000000001</v>
+      </c>
+      <c r="Q44" s="11" t="n">
+        <v>167.35</v>
+      </c>
+      <c r="R44" s="11">
+        <f>SUM(C44:Q44)</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="B45" s="2" t="n">
         <v>46306</v>
       </c>
-      <c r="C45" s="1" t="n"/>
-      <c r="D45" s="1" t="n"/>
-      <c r="E45" s="1" t="n"/>
-      <c r="F45" s="1" t="n"/>
-      <c r="G45" s="1" t="n"/>
-      <c r="H45" s="1" t="n"/>
-      <c r="I45" s="1" t="n"/>
-      <c r="J45" s="1" t="n"/>
-      <c r="K45" s="1" t="n"/>
-      <c r="L45" s="1" t="n"/>
-      <c r="M45" s="1" t="n"/>
-      <c r="N45" s="1" t="n"/>
-      <c r="O45" s="1" t="n"/>
-      <c r="P45" s="1" t="n"/>
-      <c r="Q45" s="1" t="n"/>
-      <c r="R45" s="1" t="n"/>
+      <c r="C45" s="11" t="n">
+        <v>4006.24</v>
+      </c>
+      <c r="D45" s="11" t="n">
+        <v>53.14</v>
+      </c>
+      <c r="E45" s="11" t="n">
+        <v>486.19</v>
+      </c>
+      <c r="F45" s="11" t="n">
+        <v>118.57</v>
+      </c>
+      <c r="G45" s="11" t="n">
+        <v>1098.1</v>
+      </c>
+      <c r="H45" s="11" t="n">
+        <v>1904.8</v>
+      </c>
+      <c r="I45" s="11" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="J45" s="11" t="n">
+        <v>223.27</v>
+      </c>
+      <c r="K45" s="11" t="n">
+        <v>776.96</v>
+      </c>
+      <c r="L45" s="11" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="M45" s="11" t="n">
+        <v>1043.32</v>
+      </c>
+      <c r="N45" s="11" t="n">
+        <v>12.75</v>
+      </c>
+      <c r="O45" s="11" t="n">
+        <v>684.08</v>
+      </c>
+      <c r="P45" s="11" t="n">
+        <v>632.3</v>
+      </c>
+      <c r="Q45" s="11" t="n">
+        <v>158.62</v>
+      </c>
+      <c r="R45" s="11">
+        <f>SUM(C45:Q45)</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="B46" s="2" t="n">
         <v>46307</v>
       </c>
-      <c r="C46" s="1" t="n"/>
-      <c r="D46" s="1" t="n"/>
-      <c r="E46" s="1" t="n"/>
-      <c r="F46" s="1" t="n"/>
-      <c r="G46" s="1" t="n"/>
-      <c r="H46" s="1" t="n"/>
-      <c r="I46" s="1" t="n"/>
-      <c r="J46" s="1" t="n"/>
-      <c r="K46" s="1" t="n"/>
-      <c r="L46" s="1" t="n"/>
-      <c r="M46" s="1" t="n"/>
-      <c r="N46" s="1" t="n"/>
-      <c r="O46" s="1" t="n"/>
-      <c r="P46" s="1" t="n"/>
-      <c r="Q46" s="1" t="n"/>
-      <c r="R46" s="1" t="n"/>
+      <c r="C46" s="11" t="n">
+        <v>1040.61</v>
+      </c>
+      <c r="D46" s="11" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="E46" s="11" t="n">
+        <v>60.67</v>
+      </c>
+      <c r="F46" s="11" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="G46" s="11" t="n">
+        <v>462.11</v>
+      </c>
+      <c r="H46" s="11" t="n">
+        <v>674.3200000000001</v>
+      </c>
+      <c r="I46" s="11" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="J46" s="11" t="n">
+        <v>108.02</v>
+      </c>
+      <c r="K46" s="11" t="n">
+        <v>197.92</v>
+      </c>
+      <c r="L46" s="11" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="M46" s="11" t="n">
+        <v>254.53</v>
+      </c>
+      <c r="N46" s="11" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="O46" s="11" t="n">
+        <v>247.1</v>
+      </c>
+      <c r="P46" s="11" t="n">
+        <v>197.66</v>
+      </c>
+      <c r="Q46" s="11" t="n">
+        <v>115.69</v>
+      </c>
+      <c r="R46" s="11">
+        <f>SUM(C46:Q46)</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="B47" s="2" t="n">
         <v>46308</v>
       </c>
-      <c r="C47" s="1" t="n"/>
-      <c r="D47" s="1" t="n"/>
-      <c r="E47" s="1" t="n"/>
-      <c r="F47" s="1" t="n"/>
-      <c r="G47" s="1" t="n"/>
-      <c r="H47" s="1" t="n"/>
-      <c r="I47" s="1" t="n"/>
-      <c r="J47" s="1" t="n"/>
-      <c r="K47" s="1" t="n"/>
-      <c r="L47" s="1" t="n"/>
-      <c r="M47" s="1" t="n"/>
-      <c r="N47" s="1" t="n"/>
-      <c r="O47" s="1" t="n"/>
-      <c r="P47" s="1" t="n"/>
-      <c r="Q47" s="1" t="n"/>
-      <c r="R47" s="1" t="n"/>
+      <c r="C47" s="11" t="n">
+        <v>3139.27</v>
+      </c>
+      <c r="D47" s="11" t="n">
+        <v>27.97</v>
+      </c>
+      <c r="E47" s="11" t="n">
+        <v>477.61</v>
+      </c>
+      <c r="F47" s="11" t="n">
+        <v>211.95</v>
+      </c>
+      <c r="G47" s="11" t="n">
+        <v>942.64</v>
+      </c>
+      <c r="H47" s="11" t="n">
+        <v>1553.36</v>
+      </c>
+      <c r="I47" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J47" s="11" t="n">
+        <v>175.06</v>
+      </c>
+      <c r="K47" s="11" t="n">
+        <v>583.97</v>
+      </c>
+      <c r="L47" s="11" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M47" s="11" t="n">
+        <v>809.89</v>
+      </c>
+      <c r="N47" s="11" t="n">
+        <v>19.59</v>
+      </c>
+      <c r="O47" s="11" t="n">
+        <v>547.38</v>
+      </c>
+      <c r="P47" s="11" t="n">
+        <v>484.8</v>
+      </c>
+      <c r="Q47" s="11" t="n">
+        <v>137.24</v>
+      </c>
+      <c r="R47" s="11">
+        <f>SUM(C47:Q47)</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="B48" s="2" t="n">
         <v>46309</v>
       </c>
-      <c r="C48" s="1" t="n"/>
-      <c r="D48" s="1" t="n"/>
-      <c r="E48" s="1" t="n"/>
-      <c r="F48" s="1" t="n"/>
-      <c r="G48" s="1" t="n"/>
-      <c r="H48" s="1" t="n"/>
-      <c r="I48" s="1" t="n"/>
-      <c r="J48" s="1" t="n"/>
-      <c r="K48" s="1" t="n"/>
-      <c r="L48" s="1" t="n"/>
-      <c r="M48" s="1" t="n"/>
-      <c r="N48" s="1" t="n"/>
-      <c r="O48" s="1" t="n"/>
-      <c r="P48" s="1" t="n"/>
-      <c r="Q48" s="1" t="n"/>
-      <c r="R48" s="1" t="n"/>
+      <c r="C48" s="11" t="n">
+        <v>3869.69</v>
+      </c>
+      <c r="D48" s="11" t="n">
+        <v>35.05</v>
+      </c>
+      <c r="E48" s="11" t="n">
+        <v>467.64</v>
+      </c>
+      <c r="F48" s="11" t="n">
+        <v>182.56</v>
+      </c>
+      <c r="G48" s="11" t="n">
+        <v>1122.64</v>
+      </c>
+      <c r="H48" s="11" t="n">
+        <v>1919.31</v>
+      </c>
+      <c r="I48" s="11" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="J48" s="11" t="n">
+        <v>217.33</v>
+      </c>
+      <c r="K48" s="11" t="n">
+        <v>777.11</v>
+      </c>
+      <c r="L48" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M48" s="11" t="n">
+        <v>1006.31</v>
+      </c>
+      <c r="N48" s="11" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="O48" s="11" t="n">
+        <v>708.02</v>
+      </c>
+      <c r="P48" s="11" t="n">
+        <v>633.14</v>
+      </c>
+      <c r="Q48" s="11" t="n">
+        <v>159.78</v>
+      </c>
+      <c r="R48" s="11">
+        <f>SUM(C48:Q48)</f>
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="B49" s="2" t="n">
         <v>46310</v>
       </c>
-      <c r="C49" s="1" t="n"/>
-      <c r="D49" s="1" t="n"/>
-      <c r="E49" s="1" t="n"/>
-      <c r="F49" s="1" t="n"/>
-      <c r="G49" s="1" t="n"/>
-      <c r="H49" s="1" t="n"/>
-      <c r="I49" s="1" t="n"/>
-      <c r="J49" s="1" t="n"/>
-      <c r="K49" s="1" t="n"/>
-      <c r="L49" s="1" t="n"/>
-      <c r="M49" s="1" t="n"/>
-      <c r="N49" s="1" t="n"/>
-      <c r="O49" s="1" t="n"/>
-      <c r="P49" s="1" t="n"/>
-      <c r="Q49" s="1" t="n"/>
-      <c r="R49" s="1" t="n"/>
+      <c r="C49" s="11" t="n">
+        <v>3894.02</v>
+      </c>
+      <c r="D49" s="11" t="n">
+        <v>11.96</v>
+      </c>
+      <c r="E49" s="11" t="n">
+        <v>536.78</v>
+      </c>
+      <c r="F49" s="11" t="n">
+        <v>218.23</v>
+      </c>
+      <c r="G49" s="11" t="n">
+        <v>1063.39</v>
+      </c>
+      <c r="H49" s="11" t="n">
+        <v>2062.06</v>
+      </c>
+      <c r="I49" s="11" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="J49" s="11" t="n">
+        <v>167.44</v>
+      </c>
+      <c r="K49" s="11" t="n">
+        <v>777.8</v>
+      </c>
+      <c r="L49" s="11" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="M49" s="11" t="n">
+        <v>1054.09</v>
+      </c>
+      <c r="N49" s="11" t="n">
+        <v>16.35</v>
+      </c>
+      <c r="O49" s="11" t="n">
+        <v>722.4</v>
+      </c>
+      <c r="P49" s="11" t="n">
+        <v>682.23</v>
+      </c>
+      <c r="Q49" s="11" t="n">
+        <v>136.58</v>
+      </c>
+      <c r="R49" s="11">
+        <f>SUM(C49:Q49)</f>
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="B50" s="2" t="n">
         <v>46311</v>
       </c>
-      <c r="C50" s="1" t="n"/>
-      <c r="D50" s="1" t="n"/>
-      <c r="E50" s="1" t="n"/>
-      <c r="F50" s="1" t="n"/>
-      <c r="G50" s="1" t="n"/>
-      <c r="H50" s="1" t="n"/>
-      <c r="I50" s="1" t="n"/>
-      <c r="J50" s="1" t="n"/>
-      <c r="K50" s="1" t="n"/>
-      <c r="L50" s="1" t="n"/>
-      <c r="M50" s="1" t="n"/>
-      <c r="N50" s="1" t="n"/>
-      <c r="O50" s="1" t="n"/>
-      <c r="P50" s="1" t="n"/>
-      <c r="Q50" s="1" t="n"/>
-      <c r="R50" s="1" t="n"/>
+      <c r="C50" s="11" t="n">
+        <v>3963.9</v>
+      </c>
+      <c r="D50" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" s="11" t="n">
+        <v>508.02</v>
+      </c>
+      <c r="F50" s="11" t="n">
+        <v>239.98</v>
+      </c>
+      <c r="G50" s="11" t="n">
+        <v>1121.25</v>
+      </c>
+      <c r="H50" s="11" t="n">
+        <v>2059.42</v>
+      </c>
+      <c r="I50" s="11" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="J50" s="11" t="n">
+        <v>163.63</v>
+      </c>
+      <c r="K50" s="11" t="n">
+        <v>771.25</v>
+      </c>
+      <c r="L50" s="11" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="M50" s="11" t="n">
+        <v>1038.95</v>
+      </c>
+      <c r="N50" s="11" t="n">
+        <v>19.38</v>
+      </c>
+      <c r="O50" s="11" t="n">
+        <v>727.39</v>
+      </c>
+      <c r="P50" s="11" t="n">
+        <v>668.04</v>
+      </c>
+      <c r="Q50" s="11" t="n">
+        <v>157.52</v>
+      </c>
+      <c r="R50" s="11">
+        <f>SUM(C50:Q50)</f>
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="B51" s="2" t="n">
         <v>46312</v>
       </c>
-      <c r="C51" s="1" t="n"/>
-      <c r="D51" s="1" t="n"/>
-      <c r="E51" s="1" t="n"/>
-      <c r="F51" s="1" t="n"/>
-      <c r="G51" s="1" t="n"/>
-      <c r="H51" s="1" t="n"/>
-      <c r="I51" s="1" t="n"/>
-      <c r="J51" s="1" t="n"/>
-      <c r="K51" s="1" t="n"/>
-      <c r="L51" s="1" t="n"/>
-      <c r="M51" s="1" t="n"/>
-      <c r="N51" s="1" t="n"/>
-      <c r="O51" s="1" t="n"/>
-      <c r="P51" s="1" t="n"/>
-      <c r="Q51" s="1" t="n"/>
-      <c r="R51" s="1" t="n"/>
+      <c r="C51" s="11" t="n">
+        <v>3946.82</v>
+      </c>
+      <c r="D51" s="11" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="E51" s="11" t="n">
+        <v>488.73</v>
+      </c>
+      <c r="F51" s="11" t="n">
+        <v>195.2</v>
+      </c>
+      <c r="G51" s="11" t="n">
+        <v>1064.94</v>
+      </c>
+      <c r="H51" s="11" t="n">
+        <v>1950.63</v>
+      </c>
+      <c r="I51" s="11" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="J51" s="11" t="n">
+        <v>156.54</v>
+      </c>
+      <c r="K51" s="11" t="n">
+        <v>778.4400000000001</v>
+      </c>
+      <c r="L51" s="11" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="M51" s="11" t="n">
+        <v>1044.28</v>
+      </c>
+      <c r="N51" s="11" t="n">
+        <v>23.13</v>
+      </c>
+      <c r="O51" s="11" t="n">
+        <v>721.39</v>
+      </c>
+      <c r="P51" s="11" t="n">
+        <v>612.62</v>
+      </c>
+      <c r="Q51" s="11" t="n">
+        <v>128.28</v>
+      </c>
+      <c r="R51" s="11">
+        <f>SUM(C51:Q51)</f>
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="B52" s="2" t="n">
         <v>46313</v>
       </c>
-      <c r="C52" s="1" t="n"/>
-      <c r="D52" s="1" t="n"/>
-      <c r="E52" s="1" t="n"/>
-      <c r="F52" s="1" t="n"/>
-      <c r="G52" s="1" t="n"/>
-      <c r="H52" s="1" t="n"/>
-      <c r="I52" s="1" t="n"/>
-      <c r="J52" s="1" t="n"/>
-      <c r="K52" s="1" t="n"/>
-      <c r="L52" s="1" t="n"/>
-      <c r="M52" s="1" t="n"/>
-      <c r="N52" s="1" t="n"/>
-      <c r="O52" s="1" t="n"/>
-      <c r="P52" s="1" t="n"/>
-      <c r="Q52" s="1" t="n"/>
-      <c r="R52" s="1" t="n"/>
+      <c r="C52" s="11" t="n">
+        <v>4069.79</v>
+      </c>
+      <c r="D52" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" s="11" t="n">
+        <v>518.5700000000001</v>
+      </c>
+      <c r="F52" s="11" t="n">
+        <v>258.44</v>
+      </c>
+      <c r="G52" s="11" t="n">
+        <v>1127.62</v>
+      </c>
+      <c r="H52" s="11" t="n">
+        <v>1944.28</v>
+      </c>
+      <c r="I52" s="11" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="J52" s="11" t="n">
+        <v>169.42</v>
+      </c>
+      <c r="K52" s="11" t="n">
+        <v>767.8</v>
+      </c>
+      <c r="L52" s="11" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="M52" s="11" t="n">
+        <v>1026.31</v>
+      </c>
+      <c r="N52" s="11" t="n">
+        <v>22.13</v>
+      </c>
+      <c r="O52" s="11" t="n">
+        <v>721.11</v>
+      </c>
+      <c r="P52" s="11" t="n">
+        <v>638.89</v>
+      </c>
+      <c r="Q52" s="11" t="n">
+        <v>167.71</v>
+      </c>
+      <c r="R52" s="11">
+        <f>SUM(C52:Q52)</f>
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="B53" s="2" t="n">
         <v>46314</v>
       </c>
-      <c r="C53" s="1" t="n"/>
-      <c r="D53" s="1" t="n"/>
-      <c r="E53" s="1" t="n"/>
-      <c r="F53" s="1" t="n"/>
-      <c r="G53" s="1" t="n"/>
-      <c r="H53" s="1" t="n"/>
-      <c r="I53" s="1" t="n"/>
-      <c r="J53" s="1" t="n"/>
-      <c r="K53" s="1" t="n"/>
-      <c r="L53" s="1" t="n"/>
-      <c r="M53" s="1" t="n"/>
-      <c r="N53" s="1" t="n"/>
-      <c r="O53" s="1" t="n"/>
-      <c r="P53" s="1" t="n"/>
-      <c r="Q53" s="1" t="n"/>
-      <c r="R53" s="1" t="n"/>
+      <c r="C53" s="11" t="n">
+        <v>1050.47</v>
+      </c>
+      <c r="D53" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E53" s="11" t="n">
+        <v>79.98</v>
+      </c>
+      <c r="F53" s="11" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="G53" s="11" t="n">
+        <v>429.64</v>
+      </c>
+      <c r="H53" s="11" t="n">
+        <v>661.52</v>
+      </c>
+      <c r="I53" s="11" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="J53" s="11" t="n">
+        <v>90.06999999999999</v>
+      </c>
+      <c r="K53" s="11" t="n">
+        <v>488.12</v>
+      </c>
+      <c r="L53" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M53" s="11" t="n">
+        <v>247.09</v>
+      </c>
+      <c r="N53" s="11" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="O53" s="11" t="n">
+        <v>211.38</v>
+      </c>
+      <c r="P53" s="11" t="n">
+        <v>218.48</v>
+      </c>
+      <c r="Q53" s="11" t="n">
+        <v>102.07</v>
+      </c>
+      <c r="R53" s="11">
+        <f>SUM(C53:Q53)</f>
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="B54" s="2" t="n">
         <v>46315</v>
       </c>
-      <c r="C54" s="1" t="n"/>
-      <c r="D54" s="1" t="n"/>
-      <c r="E54" s="1" t="n"/>
-      <c r="F54" s="1" t="n"/>
-      <c r="G54" s="1" t="n"/>
-      <c r="H54" s="1" t="n"/>
-      <c r="I54" s="1" t="n"/>
-      <c r="J54" s="1" t="n"/>
-      <c r="K54" s="1" t="n"/>
-      <c r="L54" s="1" t="n"/>
-      <c r="M54" s="1" t="n"/>
-      <c r="N54" s="1" t="n"/>
-      <c r="O54" s="1" t="n"/>
-      <c r="P54" s="1" t="n"/>
-      <c r="Q54" s="1" t="n"/>
-      <c r="R54" s="1" t="n"/>
+      <c r="C54" s="11" t="n">
+        <v>3157.56</v>
+      </c>
+      <c r="D54" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" s="11" t="n">
+        <v>488.71</v>
+      </c>
+      <c r="F54" s="11" t="n">
+        <v>191.14</v>
+      </c>
+      <c r="G54" s="11" t="n">
+        <v>835.13</v>
+      </c>
+      <c r="H54" s="11" t="n">
+        <v>1545.02</v>
+      </c>
+      <c r="I54" s="11" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="J54" s="11" t="n">
+        <v>140.09</v>
+      </c>
+      <c r="K54" s="11" t="n">
+        <v>585.6</v>
+      </c>
+      <c r="L54" s="11" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M54" s="11" t="n">
+        <v>822.61</v>
+      </c>
+      <c r="N54" s="11" t="n">
+        <v>11.82</v>
+      </c>
+      <c r="O54" s="11" t="n">
+        <v>515.41</v>
+      </c>
+      <c r="P54" s="11" t="n">
+        <v>485.61</v>
+      </c>
+      <c r="Q54" s="11" t="n">
+        <v>173.92</v>
+      </c>
+      <c r="R54" s="11">
+        <f>SUM(C54:Q54)</f>
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="B55" s="2" t="n">
         <v>46316</v>
       </c>
-      <c r="C55" s="1" t="n"/>
-      <c r="D55" s="1" t="n"/>
-      <c r="E55" s="1" t="n"/>
-      <c r="F55" s="1" t="n"/>
-      <c r="G55" s="1" t="n"/>
-      <c r="H55" s="1" t="n"/>
-      <c r="I55" s="1" t="n"/>
-      <c r="J55" s="1" t="n"/>
-      <c r="K55" s="1" t="n"/>
-      <c r="L55" s="1" t="n"/>
-      <c r="M55" s="1" t="n"/>
-      <c r="N55" s="1" t="n"/>
-      <c r="O55" s="1" t="n"/>
-      <c r="P55" s="1" t="n"/>
-      <c r="Q55" s="1" t="n"/>
-      <c r="R55" s="1" t="n"/>
+      <c r="C55" s="11" t="n">
+        <v>900.1900000000001</v>
+      </c>
+      <c r="D55" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" s="11" t="n">
+        <v>75.36</v>
+      </c>
+      <c r="F55" s="11" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="G55" s="11" t="n">
+        <v>279.12</v>
+      </c>
+      <c r="H55" s="11" t="n">
+        <v>415.26</v>
+      </c>
+      <c r="I55" s="11" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="J55" s="11" t="n">
+        <v>74.27</v>
+      </c>
+      <c r="K55" s="11" t="n">
+        <v>186.86</v>
+      </c>
+      <c r="L55" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M55" s="11" t="n">
+        <v>196.31</v>
+      </c>
+      <c r="N55" s="11" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="O55" s="11" t="n">
+        <v>143.02</v>
+      </c>
+      <c r="P55" s="11" t="n">
+        <v>140.63</v>
+      </c>
+      <c r="Q55" s="11" t="n">
+        <v>91.98</v>
+      </c>
+      <c r="R55" s="11">
+        <f>SUM(C55:Q55)</f>
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="B56" s="2" t="n">

</xml_diff>